<commit_message>
refactor: streamline validation logic and remove unused validators
</commit_message>
<xml_diff>
--- a/exports/resultados_validacion.xlsx
+++ b/exports/resultados_validacion.xlsx
@@ -413,33 +413,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>ID_CAT_ENCUESTAS_INFO</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>VECTOR</t>
+          <t>vector</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>TIPO</t>
+          <t>variable</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>PRECONDICION</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>ERROR</t>
+          <t>mensaje</t>
         </is>
       </c>
     </row>
@@ -454,17 +449,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>P6_4_2==0</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> P6_1==2</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>P6_4_2==0</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -479,17 +469,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>P13_1_1&gt;0</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -504,17 +489,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>((P15_1/P13_0)*100)&gt;10</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>P13_0&gt;0</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>((P15_1/P13_0)*100)&gt;10</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -529,17 +509,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>P13_1_1&gt;0</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -554,17 +529,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>P13_1_1&gt;0</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -579,17 +549,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>((P15_1/P13_0)*100)&gt;10</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>P13_0&gt;0</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>((P15_1/P13_0)*100)&gt;10</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -604,17 +569,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>P13_1_1&gt;0</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -629,17 +589,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>P13_1_1&gt;0</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>
@@ -654,17 +609,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>I</t>
+          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>P13_1_1&gt;0</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>Error de validación</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance validation process with additional columns and improved UI elements
</commit_message>
<xml_diff>
--- a/exports/resultados_validacion.xlsx
+++ b/exports/resultados_validacion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -434,7 +434,7 @@
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>mensaje</t>
+          <t>procedimiento</t>
         </is>
       </c>
     </row>
@@ -449,12 +449,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P6_4_2==0</t>
+          <t>P6_1 | P6_4_2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>06I02_2  Reconsulta con la persona informante si la persona que toma principalmente las decisiones de la empresa es mujer, ya que menciona que el porcentaje de propiedad de la empresa que está en manos de mujeres es cero. De ser necesario, corrige las variables involucradas., Acepta justificación</t>
         </is>
       </c>
     </row>
@@ -469,12 +469,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>P13_1_1 | P17_1 | P17_2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
         </is>
       </c>
     </row>
@@ -484,17 +484,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_06I01</t>
+          <t>E_ENAPROCE_15I01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t xml:space="preserve">P6_4_1==0 </t>
+          <t>P13_0 | P15_1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
         </is>
       </c>
     </row>
@@ -504,23 +504,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_15I01</t>
+          <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>((P15_1/P13_0)*100)&gt;10</t>
+          <t>P13_1_1 | P17_1 | P17_2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9002</v>
+        <v>9038</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -529,58 +529,58 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>P13_1_1 | P17_1 | P17_2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9038</v>
+        <v>9035</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_17I01</t>
+          <t>E_ENAPROCE_15I01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>P13_0 | P15_1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9035</v>
+        <v>9008</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_15I01</t>
+          <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>((P15_1/P13_0)*100)&gt;10</t>
+          <t>P13_1_1 | P17_1 | P17_2</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9008</v>
+        <v>9006</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -589,18 +589,18 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>P13_1_1 | P17_1 | P17_2</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Error de validación</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9006</v>
+        <v>9032</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
@@ -609,32 +609,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
+          <t>P13_1_1 | P17_1 | P17_2</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Error de validación</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="n">
-        <v>9032</v>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_17I01</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>(((P17_1+P17_2)/P13_1_1)/12 &lt; 1050 or ((P17_1+P17_2)/P13_1_1)/12 &gt; 60000)</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>Error de validación</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add main application logic and configuration files
- Implemented the main application in main.py using customtkinter for the UI.
- Created a main.spec file for packaging the application with PyInstaller.
- Added a new Excel file for data handling.
</commit_message>
<xml_diff>
--- a/exports/resultados_validacion.xlsx
+++ b/exports/resultados_validacion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,17 +424,17 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>vector</t>
+          <t>Nombre Vector</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>variable</t>
+          <t>Variables Involucradas</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>procedimiento</t>
+          <t>Procedimiento</t>
         </is>
       </c>
     </row>
@@ -460,47 +460,47 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>9007</v>
+        <v>9012</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_17I01</t>
+          <t>E_ENAPROCE_P5_9X</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
+          <t>P5_9X</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+          <t>Es parecido a Persona fundadora)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9002</v>
+        <v>9014</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_15I01</t>
+          <t>E_ENAPROCE_P5_9X</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>P13_0 | P15_1</t>
+          <t>P5_9X</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
+          <t>Es parecido a Persona fundadora)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>9002</v>
+        <v>9007</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -520,101 +520,761 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9038</v>
+        <v>9007</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_17I01</t>
+          <t>E_ENAPROCE_P5_9X</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
+          <t>P5_9X</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+          <t>Es parecido a Persona fundadora)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9035</v>
+        <v>9039</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_15I01</t>
+          <t>E_ENAPROCE_P3_19X</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>P13_0 | P15_1</t>
+          <t>P3_19X</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
+          <t>Es parecido a Servicios públicos)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9008</v>
+        <v>9039</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_17I01</t>
+          <t>E_ENAPROCE_P5_9X</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
+          <t>P5_9X</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+          <t>Es parecido a Persona fundadora)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9006</v>
+        <v>9002</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_17I01</t>
+          <t>E_ENAPROCE_15I01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
+          <t>P13_0 | P15_1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_17I01</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>P13_1_1 | P17_1 | P17_2</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9002</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P2_9X</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>P2_9X</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Es parecido a Propios)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>9002</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P3_19X</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>P3_19X</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Es parecido a Accesos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>9002</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Es parecido a Persona fundadora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>9038</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_17I01</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>P13_1_1 | P17_1 | P17_2</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>9038</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Es parecido a Individuos(as) privados(as))</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_15I01</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>P13_0 | P15_1</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P2_9X</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>P2_9X</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Texto basura: hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P4_9X</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>P4_9X</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Texto basura: ooooooooooooooooooooooooooooooooooooooooooooooooooooooooooo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Es parecido a Persona fundadora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P9_9X</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>P9_9X</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P16_9X</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>P16_9X</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P18_9X</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>P18_9X</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Texto basura: uuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuu</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P38_9X</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>P38_9X</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Texto basura: jjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjj</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P46_9X</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>P46_9X</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Texto basura: ñlllllllllllllllllllllllllllllllllllllllllllllllllllllllllll</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P52_9X</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>P52_9X</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P54_9X</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>P54_9X</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Texto basura: iiiiiiiiiiiiiiiiiiiidddddddddddddddddddddddddddddddddddddddd</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P55_3_19X</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>P55_3_19X</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Texto basura: sssssssssssssssssssssssssss</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P55_4_9X</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>P55_4_9X</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Texto basura: dddddddddddddddddddddddddddddddddddddd</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P58_19X</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>P58_19X</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Texto basura: oooooooooooooooooooooooooooooooooooooooooooooooooooooooooooo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P65_9X</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>P65_9X</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Texto basura: aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P73_19X</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>P73_19X</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Texto basura: aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaabb</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P76_9X</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>P76_9X</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Texto basura: uuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuu</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P78_9X</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>P78_9X</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Texto basura: hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>9035</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P81_19X</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>P81_19X</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Texto basura: cccccccccccccccccccccccccccccccccccccccccccccccccccccr</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>9008</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_17I01</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>P13_1_1 | P17_1 | P17_2</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>9008</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Es parecido a Persona fundadora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>9006</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_17I01</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>P13_1_1 | P17_1 | P17_2</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>9006</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Es parecido a Persona fundadora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>9031</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Es parecido a Persona fundadora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>9034</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P3_19X</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>P3_19X</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Es parecido a Propietario del inmueble)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>9034</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Es parecido a Persona fundadora)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
         <v>9032</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>P13_1_1 | P17_1 | P17_2</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="D42" t="inlineStr">
         <is>
           <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>9032</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>E_ENAPROCE_P5_9X</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>P5_9X</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Es parecido a Persona fundadora)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: enhance validation UI with detailed error display and improved table structure
</commit_message>
<xml_diff>
--- a/exports/resultados_validacion.xlsx
+++ b/exports/resultados_validacion.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D43"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,58 +449,58 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>P6_1 | P6_4_2</t>
+          <t>P6_1, P6_4_2</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>06I02_2  Reconsulta con la persona informante si la persona que toma principalmente las decisiones de la empresa es mujer, ya que menciona que el porcentaje de propiedad de la empresa que está en manos de mujeres es cero. De ser necesario, corrige las variables involucradas., Acepta justificación</t>
+          <t>06I02_2 Reconsulta con la persona informante si la persona que toma principalmente las decisiones de la empresa es mujer, ya que menciona que el porcentaje de propiedad de la empresa que está en manos de mujeres es cero. De ser necesario, corrige las variables involucradas. Acepta justificación</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>9012</v>
+        <v>9007</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P5_9X</t>
+          <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>P5_9X</t>
+          <t>P13_1_1, P17_1, P17_2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Es parecido a Persona fundadora)</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año. Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>9014</v>
+        <v>9002</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P5_9X</t>
+          <t>E_ENAPROCE_15I01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>P5_9X</t>
+          <t>P13_0, P15_1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Es parecido a Persona fundadora)</t>
+          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025. Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>9007</v>
+        <v>9002</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -509,212 +509,212 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
+          <t>P13_1_1, P17_1, P17_2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año. Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9007</v>
+        <v>9038</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P5_9X</t>
+          <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>P5_9X</t>
+          <t>P13_1_1, P17_1, P17_2</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Es parecido a Persona fundadora)</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año. Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>9039</v>
+        <v>9035</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P3_19X</t>
+          <t>E_ENAPROCE_15I01</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>P3_19X</t>
+          <t>P13_0, P15_1</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Es parecido a Servicios públicos)</t>
+          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025. Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>9039</v>
+        <v>9035</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P5_9X</t>
+          <t>E_ENAPROCE_02O01</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>P5_9X</t>
+          <t>P2_9X</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Es parecido a Persona fundadora)</t>
+          <t>Texto basura: hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9002</v>
+        <v>9035</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_15I01</t>
+          <t>E_ENAPROCE_04O01</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>P13_0 | P15_1</t>
+          <t>P4_9X</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
+          <t>Texto basura: ooooooooooooooooooooooooooooooooooooooooooooooooooooooooooo</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>9002</v>
+        <v>9035</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_17I01</t>
+          <t>E_ENAPROCE_09O01</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
+          <t>P9_9X</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>9002</v>
+        <v>9035</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P2_9X</t>
+          <t>E_ENAPROCE_16O01</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>P2_9X</t>
+          <t>P16_9X</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Es parecido a Propios)</t>
+          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>9002</v>
+        <v>9035</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P3_19X</t>
+          <t>E_ENAPROCE_18O01</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>P3_19X</t>
+          <t>P18_9X</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Es parecido a Accesos)</t>
+          <t>Texto basura: uuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuu</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>9002</v>
+        <v>9035</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P5_9X</t>
+          <t>E_ENAPROCE_38O01</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>P5_9X</t>
+          <t>P38_9X</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Es parecido a Persona fundadora)</t>
+          <t>Texto basura: jjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjj</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>9038</v>
+        <v>9035</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_17I01</t>
+          <t>E_ENAPROCE_46O01</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
+          <t>P46_9X</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
+          <t>Texto basura: ñlllllllllllllllllllllllllllllllllllllllllllllllllllllllllll</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>9038</v>
+        <v>9035</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P5_9X</t>
+          <t>E_ENAPROCE_52O01</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>P5_9X</t>
+          <t>P52_9X</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Es parecido a Individuos(as) privados(as))</t>
+          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
         </is>
       </c>
     </row>
@@ -724,17 +724,17 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_15I01</t>
+          <t>E_ENAPROCE_54O01</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>P13_0 | P15_1</t>
+          <t>P54_9X</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>15I01_2 Reconsulta con la persona informante el motivo por el cual el porcentaje de personal por nivel de estudios (sin instrucción) es mayor al 10 % del total del personal durante el año 2025., Acepta justificación.</t>
+          <t>Texto basura: iiiiiiiiiiiiiiiiiiiidddddddddddddddddddddddddddddddddddddddd</t>
         </is>
       </c>
     </row>
@@ -744,17 +744,17 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P2_9X</t>
+          <t>E_ENAPROCE_55O01</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>P2_9X</t>
+          <t>P55_3_19X</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Texto basura: hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</t>
+          <t>Texto basura: sssssssssssssssssssssssssss</t>
         </is>
       </c>
     </row>
@@ -764,17 +764,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P4_9X</t>
+          <t>E_ENAPROCE_55O01</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>P4_9X</t>
+          <t>P55_4_9X</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Texto basura: ooooooooooooooooooooooooooooooooooooooooooooooooooooooooooo</t>
+          <t>Texto basura: dddddddddddddddddddddddddddddddddddddd</t>
         </is>
       </c>
     </row>
@@ -784,17 +784,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P5_9X</t>
+          <t>E_ENAPROCE_58O01</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>P5_9X</t>
+          <t>P58_19X</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Es parecido a Persona fundadora)</t>
+          <t>Texto basura: oooooooooooooooooooooooooooooooooooooooooooooooooooooooooooo</t>
         </is>
       </c>
     </row>
@@ -804,17 +804,17 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P9_9X</t>
+          <t>E_ENAPROCE_65O01</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>P9_9X</t>
+          <t>P65_9X</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
+          <t>Texto basura: aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
         </is>
       </c>
     </row>
@@ -824,17 +824,17 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P16_9X</t>
+          <t>E_ENAPROCE_73O01</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>P16_9X</t>
+          <t>P73_19X</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
+          <t>Texto basura: aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaabb</t>
         </is>
       </c>
     </row>
@@ -844,17 +844,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P18_9X</t>
+          <t>E_ENAPROCE_76O01</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>P18_9X</t>
+          <t>P76_9X</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Texto basura: uuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuu</t>
+          <t>Texto basura: uuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuu</t>
         </is>
       </c>
     </row>
@@ -864,17 +864,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P38_9X</t>
+          <t>E_ENAPROCE_78O01</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>P38_9X</t>
+          <t>P78_9X</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Texto basura: jjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjjj</t>
+          <t>Texto basura: hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</t>
         </is>
       </c>
     </row>
@@ -884,397 +884,77 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P46_9X</t>
+          <t>E_ENAPROCE_81O01</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>P46_9X</t>
+          <t>P81_19X</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Texto basura: ñlllllllllllllllllllllllllllllllllllllllllllllllllllllllllll</t>
+          <t>Texto basura: cccccccccccccccccccccccccccccccccccccccccccccccccccccr</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>9035</v>
+        <v>9008</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P52_9X</t>
+          <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>P52_9X</t>
+          <t>P13_1_1, P17_1, P17_2</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Texto basura: kkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkkk</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año. Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>9035</v>
+        <v>9006</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P54_9X</t>
+          <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>P54_9X</t>
+          <t>P13_1_1, P17_1, P17_2</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Texto basura: iiiiiiiiiiiiiiiiiiiidddddddddddddddddddddddddddddddddddddddd</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año. Acepta justificación.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>9035</v>
+        <v>9032</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>E_ENAPROCE_P55_3_19X</t>
+          <t>E_ENAPROCE_17I01</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>P55_3_19X</t>
+          <t>P13_1_1, P17_1, P17_2</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Texto basura: sssssssssssssssssssssssssss</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>9035</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P55_4_9X</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>P55_4_9X</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>Texto basura: dddddddddddddddddddddddddddddddddddddd</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>9035</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P58_19X</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>P58_19X</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>Texto basura: oooooooooooooooooooooooooooooooooooooooooooooooooooooooooooo</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>9035</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P65_9X</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>P65_9X</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>Texto basura: aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaa</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>9035</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P73_19X</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>P73_19X</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>Texto basura: aaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaaabb</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>9035</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P76_9X</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>P76_9X</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Texto basura: uuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuuu</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>9035</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P78_9X</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>P78_9X</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>Texto basura: hhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhhh</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>9035</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P81_19X</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>P81_19X</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>Texto basura: cccccccccccccccccccccccccccccccccccccccccccccccccccccr</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>9008</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_17I01</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>9008</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P5_9X</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>P5_9X</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Es parecido a Persona fundadora)</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>9006</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_17I01</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>9006</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P5_9X</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>P5_9X</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Es parecido a Persona fundadora)</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>9031</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P5_9X</t>
-        </is>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>P5_9X</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>Es parecido a Persona fundadora)</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>9034</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P3_19X</t>
-        </is>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>P3_19X</t>
-        </is>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Es parecido a Propietario del inmueble)</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>9034</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P5_9X</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>P5_9X</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Es parecido a Persona fundadora)</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>9032</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_17I01</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>P13_1_1 | P17_1 | P17_2</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año., Acepta justificación.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>9032</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>E_ENAPROCE_P5_9X</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>P5_9X</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Es parecido a Persona fundadora)</t>
+          <t>17I01_2 Reconsulta con la persona informante la cantidad correcta de las remuneraciones anuales pagadas, así como el personal ocupado dependiente de la razón social durante el año 2025. Asimismo, verifica que las remuneraciones se encuentren expresadas en pesos, ya que los montos reportados podrían resultar muy bajos o muy altos para el año 2025, así como el número de meses laborados por la empresa en dicho año. Acepta justificación.</t>
         </is>
       </c>
     </row>

</xml_diff>